<commit_message>
close to final 2.25
</commit_message>
<xml_diff>
--- a/results/02-2026/no-tariffs/beta/contributions-02-2026.xlsx
+++ b/results/02-2026/no-tariffs/beta/contributions-02-2026.xlsx
@@ -22360,13 +22360,13 @@
         <v>-0.0289055700739013</v>
       </c>
       <c r="F224" t="n">
-        <v>-0.535864414744887</v>
+        <v>-0.0727930741855072</v>
       </c>
       <c r="G224" t="n">
         <v>-0.014530714174193</v>
       </c>
       <c r="H224" t="n">
-        <v>0.126456632364786</v>
+        <v>-0.0108481072617925</v>
       </c>
       <c r="I224" t="n">
         <v>0.233931922438709</v>
@@ -22423,19 +22423,19 @@
         <v>-0.261464773606026</v>
       </c>
       <c r="AA224" t="n">
-        <v>-0.175063269328131</v>
+        <v>0.149212846958388</v>
       </c>
       <c r="AB224" t="n">
         <v>0.400499987399627</v>
       </c>
       <c r="AC224" t="n">
-        <v>0.226162205946252</v>
+        <v>0.549094129176975</v>
       </c>
       <c r="AD224" t="n">
-        <v>0.22429613644264</v>
+        <v>0.547228059673362</v>
       </c>
       <c r="AE224" t="n">
-        <v>-0.0984604793437247</v>
+        <v>-0.0177274985360441</v>
       </c>
     </row>
     <row r="225">
@@ -22455,13 +22455,13 @@
         <v>0.0154321783725609</v>
       </c>
       <c r="F225" t="n">
-        <v>-0.477219622900714</v>
+        <v>0.0638754327850785</v>
       </c>
       <c r="G225" t="n">
         <v>-0.0219353935221326</v>
       </c>
       <c r="H225" t="n">
-        <v>0.0126381468949599</v>
+        <v>0.0143422374092909</v>
       </c>
       <c r="I225" t="n">
         <v>0.142848301801328</v>
@@ -22518,19 +22518,19 @@
         <v>0.462105508553894</v>
       </c>
       <c r="AA225" t="n">
-        <v>-0.324072112830468</v>
+        <v>0.217858967621791</v>
       </c>
       <c r="AB225" t="n">
         <v>0.398712351775537</v>
       </c>
       <c r="AC225" t="n">
-        <v>0.0759956405318908</v>
+        <v>0.615659282515708</v>
       </c>
       <c r="AD225" t="n">
-        <v>-1.14696133140951</v>
+        <v>-0.607297689425689</v>
       </c>
       <c r="AE225" t="n">
-        <v>-0.512922377869266</v>
+        <v>-0.297273486565631</v>
       </c>
     </row>
     <row r="226">
@@ -22550,13 +22550,13 @@
         <v>-0.188450438947078</v>
       </c>
       <c r="F226" t="n">
-        <v>-0.16023109196327</v>
+        <v>0.148446852745259</v>
       </c>
       <c r="G226" t="n">
         <v>-0.00506423037529374</v>
       </c>
       <c r="H226" t="n">
-        <v>0.0185376543451162</v>
+        <v>0.0202329326727563</v>
       </c>
       <c r="I226" t="n">
         <v>0.31528095571367</v>
@@ -22613,19 +22613,19 @@
         <v>-0.137509049814841</v>
       </c>
       <c r="AA226" t="n">
-        <v>0.183980310304984</v>
+        <v>0.493222274248671</v>
       </c>
       <c r="AB226" t="n">
         <v>0.468605507989397</v>
       </c>
       <c r="AC226" t="n">
-        <v>0.71167271683087</v>
+        <v>1.01937856347546</v>
       </c>
       <c r="AD226" t="n">
-        <v>2.5198390274119</v>
+        <v>2.82754487405649</v>
       </c>
       <c r="AE226" t="n">
-        <v>0.290895719164186</v>
+        <v>0.583471072128967</v>
       </c>
     </row>
     <row r="227">
@@ -22645,13 +22645,13 @@
         <v>-0.175946814023728</v>
       </c>
       <c r="F227" t="n">
-        <v>-0.0995165316787522</v>
+        <v>0.16326367649741</v>
       </c>
       <c r="G227" t="n">
         <v>-0.00747752072963209</v>
       </c>
       <c r="H227" t="n">
-        <v>0.0204607145182782</v>
+        <v>0.0220396079445972</v>
       </c>
       <c r="I227" t="n">
         <v>0.251293432943367</v>
@@ -22708,19 +22708,19 @@
         <v>-0.0917213099292404</v>
       </c>
       <c r="AA227" t="n">
-        <v>0.177256923604722</v>
+        <v>0.44084386790875</v>
       </c>
       <c r="AB227" t="n">
         <v>0.257254349518803</v>
       </c>
       <c r="AC227" t="n">
-        <v>0.494030937613784</v>
+        <v>0.756903053308723</v>
       </c>
       <c r="AD227" t="n">
-        <v>0.0160537096492648</v>
+        <v>0.278925825344203</v>
       </c>
       <c r="AE227" t="n">
-        <v>0.403306885523575</v>
+        <v>0.761600267412092</v>
       </c>
     </row>
     <row r="228">
@@ -22740,13 +22740,13 @@
         <v>-0.174807656662485</v>
       </c>
       <c r="F228" t="n">
-        <v>-0.147974511414025</v>
+        <v>0.111256487568322</v>
       </c>
       <c r="G228" t="n">
         <v>-0.00938410867798814</v>
       </c>
       <c r="H228" t="n">
-        <v>0.0303528561543755</v>
+        <v>0.0318778727871187</v>
       </c>
       <c r="I228" t="n">
         <v>0.0778533087561076</v>
@@ -22803,19 +22803,19 @@
         <v>-0.138678614163938</v>
       </c>
       <c r="AA228" t="n">
-        <v>-0.0381310407669006</v>
+        <v>0.222321411648103</v>
       </c>
       <c r="AB228" t="n">
         <v>0.369609009894661</v>
       </c>
       <c r="AC228" t="n">
-        <v>0.391626997522706</v>
+        <v>0.651061119280384</v>
       </c>
       <c r="AD228" t="n">
-        <v>-0.0344933113116735</v>
+        <v>0.224940810446004</v>
       </c>
       <c r="AE228" t="n">
-        <v>0.338609523584997</v>
+        <v>0.681028455105252</v>
       </c>
     </row>
     <row r="229">
@@ -22835,13 +22835,13 @@
         <v>-0.198325825071049</v>
       </c>
       <c r="F229" t="n">
-        <v>-0.131758952366428</v>
+        <v>0.124674268006865</v>
       </c>
       <c r="G229" t="n">
         <v>-0.00497152729214828</v>
       </c>
       <c r="H229" t="n">
-        <v>0.0271802728302014</v>
+        <v>0.0286269232710731</v>
       </c>
       <c r="I229" t="n">
         <v>-0.0522398538563686</v>
@@ -22898,19 +22898,19 @@
         <v>-0.139460435168507</v>
       </c>
       <c r="AA229" t="n">
-        <v>-0.150144116727953</v>
+        <v>0.107784459022748</v>
       </c>
       <c r="AB229" t="n">
         <v>0.329945563885235</v>
       </c>
       <c r="AC229" t="n">
-        <v>0.240326915355869</v>
+        <v>0.497352631544775</v>
       </c>
       <c r="AD229" t="n">
-        <v>-0.0691999386579741</v>
+        <v>0.187825777530931</v>
       </c>
       <c r="AE229" t="n">
-        <v>0.60804987177288</v>
+        <v>0.879809321844407</v>
       </c>
     </row>
     <row r="230">
@@ -22930,13 +22930,13 @@
         <v>-0.184705112342636</v>
       </c>
       <c r="F230" t="n">
-        <v>-0.384339553800794</v>
+        <v>-0.130027867040536</v>
       </c>
       <c r="G230" t="n">
         <v>-0.00480207754633699</v>
       </c>
       <c r="H230" t="n">
-        <v>0.0369469044815052</v>
+        <v>0.0383482272632666</v>
       </c>
       <c r="I230" t="n">
         <v>-0.266610705133464</v>
@@ -22993,19 +22993,19 @@
         <v>-0.138670697334917</v>
       </c>
       <c r="AA230" t="n">
-        <v>-0.607867404837882</v>
+        <v>-0.351546934344287</v>
       </c>
       <c r="AB230" t="n">
         <v>0.183800587850174</v>
       </c>
       <c r="AC230" t="n">
-        <v>-0.36287882629361</v>
+        <v>-0.107058987141543</v>
       </c>
       <c r="AD230" t="n">
-        <v>-0.666171939200639</v>
+        <v>-0.410352100048572</v>
       </c>
       <c r="AE230" t="n">
-        <v>-0.188452869880255</v>
+        <v>0.0703350783181416</v>
       </c>
     </row>
     <row r="231">
@@ -23025,13 +23025,13 @@
         <v>-0.179276164652479</v>
       </c>
       <c r="F231" t="n">
-        <v>-0.246754030865279</v>
+        <v>0.0048824127824564</v>
       </c>
       <c r="G231" t="n">
         <v>-0.000572507778167652</v>
       </c>
       <c r="H231" t="n">
-        <v>0.0437430886635974</v>
+        <v>0.0451055510185345</v>
       </c>
       <c r="I231" t="n">
         <v>-0.3634641147857</v>
@@ -23088,19 +23088,19 @@
         <v>-0.134937386629759</v>
       </c>
       <c r="AA231" t="n">
-        <v>-0.557348883426182</v>
+        <v>-0.303514344782022</v>
       </c>
       <c r="AB231" t="n">
         <v>0.122874806962723</v>
       </c>
       <c r="AC231" t="n">
-        <v>-0.373744234997763</v>
+        <v>-0.120241911022423</v>
       </c>
       <c r="AD231" t="n">
-        <v>-0.654496079216422</v>
+        <v>-0.400993755241083</v>
       </c>
       <c r="AE231" t="n">
-        <v>-0.356090317096677</v>
+        <v>-0.0996448168281799</v>
       </c>
     </row>
     <row r="232">
@@ -23120,13 +23120,13 @@
         <v>-0.186499084275908</v>
       </c>
       <c r="F232" t="n">
-        <v>0.00909403730935971</v>
+        <v>0.0532998757560604</v>
       </c>
       <c r="G232" t="n">
         <v>0.00267963321166658</v>
       </c>
       <c r="H232" t="n">
-        <v>0.0391985786873209</v>
+        <v>0.0405304762437432</v>
       </c>
       <c r="I232" t="n">
         <v>-0.386048848321532</v>
@@ -23183,19 +23183,19 @@
         <v>-0.143839529777795</v>
       </c>
       <c r="AA232" t="n">
-        <v>-0.324871708306209</v>
+        <v>-0.279172169402532</v>
       </c>
       <c r="AB232" t="n">
         <v>0.0806333520828782</v>
       </c>
       <c r="AC232" t="n">
-        <v>-0.243959322514447</v>
+        <v>-0.198299015742875</v>
       </c>
       <c r="AD232" t="n">
-        <v>-0.538828145811263</v>
+        <v>-0.493167839039691</v>
       </c>
       <c r="AE232" t="n">
-        <v>-0.482174025721574</v>
+        <v>-0.279171979199603</v>
       </c>
     </row>
     <row r="233">
@@ -23215,13 +23215,13 @@
         <v>-0.182999695185691</v>
       </c>
       <c r="F233" t="n">
-        <v>0.0660408374629679</v>
+        <v>0.0690480099129439</v>
       </c>
       <c r="G233" t="n">
         <v>0.0111112928611555</v>
       </c>
       <c r="H233" t="n">
-        <v>0.0438721202272216</v>
+        <v>0.0451727040080531</v>
       </c>
       <c r="I233" t="n">
         <v>-0.42829519823617</v>
@@ -23278,19 +23278,19 @@
         <v>-0.14175729010882</v>
       </c>
       <c r="AA233" t="n">
-        <v>-0.295810655907873</v>
+        <v>-0.291486614785071</v>
       </c>
       <c r="AB233" t="n">
         <v>0.00955802153616681</v>
       </c>
       <c r="AC233" t="n">
-        <v>-0.286222484080017</v>
+        <v>-0.28189888345425</v>
       </c>
       <c r="AD233" t="n">
-        <v>-0.648178677971871</v>
+        <v>-0.643855077346103</v>
       </c>
       <c r="AE233" t="n">
-        <v>-0.626918710550049</v>
+        <v>-0.487092192918862</v>
       </c>
     </row>
     <row r="234">
@@ -23310,13 +23310,13 @@
         <v>-10.7880078888846</v>
       </c>
       <c r="F234" t="n">
-        <v>7.79870116289761</v>
+        <v>7.30188606225117</v>
       </c>
       <c r="G234" t="n">
         <v>3.96422368180105</v>
       </c>
       <c r="H234" t="n">
-        <v>0.20912659000582</v>
+        <v>0.21039758636219</v>
       </c>
       <c r="I234" t="n">
         <v>-0.616271158703167</v>
@@ -23373,19 +23373,19 @@
         <v>-9.28684364027715</v>
       </c>
       <c r="AA234" t="n">
-        <v>11.1431831852029</v>
+        <v>10.6675425975116</v>
       </c>
       <c r="AB234" t="n">
         <v>-16.5792574406224</v>
       </c>
       <c r="AC234" t="n">
-        <v>-3.4757549119512</v>
+        <v>-4.03695405109655</v>
       </c>
       <c r="AD234" t="n">
-        <v>-20.6449502511878</v>
+        <v>-21.2061493903331</v>
       </c>
       <c r="AE234" t="n">
-        <v>-5.62161328854684</v>
+        <v>-5.68604151549</v>
       </c>
     </row>
     <row r="235">
@@ -23405,13 +23405,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F235" t="n">
-        <v>7.68816499631454</v>
+        <v>7.19579524664582</v>
       </c>
       <c r="G235" t="n">
         <v>3.92261749916195</v>
       </c>
       <c r="H235" t="n">
-        <v>0.204889875640751</v>
+        <v>0.206134851818053</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
@@ -23468,19 +23468,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA235" t="n">
-        <v>11.5313850134348</v>
+        <v>11.0629705376649</v>
       </c>
       <c r="AB235" t="n">
         <v>-16.3587463870899</v>
       </c>
       <c r="AC235" t="n">
-        <v>-2.82011826600563</v>
+        <v>-3.3719833451261</v>
       </c>
       <c r="AD235" t="n">
         <v>0</v>
       </c>
       <c r="AE235" t="n">
-        <v>-5.45798926874273</v>
+        <v>-5.58579307667973</v>
       </c>
     </row>
     <row r="236">
@@ -23500,13 +23500,13 @@
         <v>#NUM!</v>
       </c>
       <c r="F236" t="n">
-        <v>3.84634964461414</v>
+        <v>3.59263887813295</v>
       </c>
       <c r="G236" t="n">
         <v>1.96595109090008</v>
       </c>
       <c r="H236" t="n">
-        <v>0.0987120125842267</v>
+        <v>0.217161929128092</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -23563,19 +23563,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA236" t="n">
-        <v>5.89072576047698</v>
+        <v>5.75424774342785</v>
       </c>
       <c r="AB236" t="n">
         <v>-16.1873864198053</v>
       </c>
       <c r="AC236" t="n">
-        <v>-9.29276672702576</v>
+        <v>-9.45277019231331</v>
       </c>
       <c r="AD236" t="n">
         <v>0</v>
       </c>
       <c r="AE236" t="n">
-        <v>-5.32328223228992</v>
+        <v>-5.46250111691981</v>
       </c>
     </row>
     <row r="237">
@@ -23595,7 +23595,7 @@
         <v>#NUM!</v>
       </c>
       <c r="F237" t="n">
-        <v>3.79390792980619</v>
+        <v>3.54234383593418</v>
       </c>
       <c r="G237" t="n">
         <v>1.94596960278224</v>
@@ -23658,19 +23658,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA237" t="n">
-        <v>5.90623609683258</v>
+        <v>5.66070442329456</v>
       </c>
       <c r="AB237" t="n">
         <v>-15.8787229378713</v>
       </c>
       <c r="AC237" t="n">
-        <v>-8.98383381140668</v>
+        <v>-9.27092919587027</v>
       </c>
       <c r="AD237" t="n">
         <v>0</v>
       </c>
       <c r="AE237" t="n">
-        <v>-5.16123756279695</v>
+        <v>-5.30153734758329</v>
       </c>
     </row>
     <row r="238">
@@ -23690,7 +23690,7 @@
         <v>#NUM!</v>
       </c>
       <c r="F238" t="n">
-        <v>3.88930084058381</v>
+        <v>3.63985838142206</v>
       </c>
       <c r="G238" t="n">
         <v>1.92748364341896</v>
@@ -23753,19 +23753,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA238" t="n">
-        <v>5.97382184305073</v>
+        <v>5.73028449008651</v>
       </c>
       <c r="AB238" t="n">
         <v>-0.0800165048843785</v>
       </c>
       <c r="AC238" t="n">
-        <v>5.89897067713867</v>
+        <v>5.65522046060019</v>
       </c>
       <c r="AD238" t="n">
         <v>0</v>
       </c>
       <c r="AE238" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="239">
@@ -23785,7 +23785,7 @@
         <v>#NUM!</v>
       </c>
       <c r="F239" t="n">
-        <v>3.84053019114867</v>
+        <v>3.5928905091504</v>
       </c>
       <c r="G239" t="n">
         <v>1.90830322592525</v>
@@ -23848,19 +23848,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA239" t="n">
-        <v>5.89915473210064</v>
+        <v>5.65729755159019</v>
       </c>
       <c r="AB239" t="n">
         <v>-0.0633243865773807</v>
       </c>
       <c r="AC239" t="n">
-        <v>5.83986490558634</v>
+        <v>5.59784054320732</v>
       </c>
       <c r="AD239" t="n">
         <v>0</v>
       </c>
       <c r="AE239" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="240">
@@ -23880,7 +23880,7 @@
         <v>#NUM!</v>
       </c>
       <c r="F240" t="n">
-        <v>3.79417525330108</v>
+        <v>3.54820591686687</v>
       </c>
       <c r="G240" t="n">
         <v>1.89080344360167</v>
@@ -23943,19 +23943,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA240" t="n">
-        <v>5.82897282863262</v>
+        <v>5.58867225006401</v>
       </c>
       <c r="AB240" t="n">
         <v>-0.0680433559075148</v>
       </c>
       <c r="AC240" t="n">
-        <v>5.76520960044907</v>
+        <v>5.52473070973455</v>
       </c>
       <c r="AD240" t="n">
         <v>0</v>
       </c>
       <c r="AE240" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="241">
@@ -23975,7 +23975,7 @@
         <v>#NUM!</v>
       </c>
       <c r="F241" t="n">
-        <v>3.74732815876936</v>
+        <v>3.50304973494493</v>
       </c>
       <c r="G241" t="n">
         <v>1.87328595039581</v>
@@ -24038,19 +24038,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA241" t="n">
-        <v>5.76922428351158</v>
+        <v>5.53053265493381</v>
       </c>
       <c r="AB241" t="n">
         <v>-0.0600433233806149</v>
       </c>
       <c r="AC241" t="n">
-        <v>5.71291672333632</v>
+        <v>5.47406892112181</v>
       </c>
       <c r="AD241" t="n">
         <v>0</v>
       </c>
       <c r="AE241" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="242">
@@ -24145,7 +24145,7 @@
         <v>0</v>
       </c>
       <c r="AE242" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="243">
@@ -24240,7 +24240,7 @@
         <v>0</v>
       </c>
       <c r="AE243" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="244">
@@ -24335,7 +24335,7 @@
         <v>0</v>
       </c>
       <c r="AE244" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245">
@@ -24430,7 +24430,7 @@
         <v>0</v>
       </c>
       <c r="AE245" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="246">
@@ -24525,7 +24525,7 @@
         <v>0</v>
       </c>
       <c r="AE246" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="247">
@@ -24620,7 +24620,7 @@
         <v>0</v>
       </c>
       <c r="AE247" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248">
@@ -24715,7 +24715,7 @@
         <v>0</v>
       </c>
       <c r="AE248" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="249">
@@ -24810,7 +24810,7 @@
         <v>0</v>
       </c>
       <c r="AE249" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250">
@@ -24905,7 +24905,7 @@
         <v>0</v>
       </c>
       <c r="AE250" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="251">
@@ -25000,7 +25000,7 @@
         <v>0</v>
       </c>
       <c r="AE251" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="252">
@@ -25095,7 +25095,7 @@
         <v>0</v>
       </c>
       <c r="AE252" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="253">
@@ -25190,7 +25190,7 @@
         <v>0</v>
       </c>
       <c r="AE253" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="254">
@@ -25285,7 +25285,7 @@
         <v>0</v>
       </c>
       <c r="AE254" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="255">
@@ -25380,7 +25380,7 @@
         <v>0</v>
       </c>
       <c r="AE255" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="256">
@@ -25475,7 +25475,7 @@
         <v>0</v>
       </c>
       <c r="AE256" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="257">
@@ -25570,7 +25570,7 @@
         <v>0</v>
       </c>
       <c r="AE257" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="258">
@@ -25665,7 +25665,7 @@
         <v>0</v>
       </c>
       <c r="AE258" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="259">
@@ -25760,7 +25760,7 @@
         <v>0</v>
       </c>
       <c r="AE259" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="260">
@@ -25855,7 +25855,7 @@
         <v>0</v>
       </c>
       <c r="AE260" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>